<commit_message>
ADNOCLS: bibliography delivered, and impossible dates made impossible
Every one of the 591 inputs is rendered in the register, grouped by research
layer, with 15 judgements each carrying what would overturn it, 7 negative
results and 3 source discrepancies.

Twelve quarter-tag dates were not calendar dates at all — the construction
produced 30 June as the 31st. They are corrected, and compute.py now parses
every input date before it writes, so a date nobody could look up fails the
build rather than reaching a reader.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FX6uP9o59mB1WpgL9CePqV
</commit_message>
<xml_diff>
--- a/engine/adnocls_study/ADNOCLS_Valuation_Model_09082026_public.xlsx
+++ b/engine/adnocls_study/ADNOCLS_Valuation_Model_09082026_public.xlsx
@@ -7837,7 +7837,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H117"/>
+  <dimension ref="A1:H112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -9225,51 +9225,7 @@
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="11" t="inlineStr">
-        <is>
-          <t>The realised vessel sale — direct evidence on carrying values</t>
-        </is>
-      </c>
-      <c r="B112" s="14" t="n"/>
-      <c r="C112" s="14" t="n"/>
-      <c r="D112" s="14" t="n"/>
-      <c r="E112" s="14" t="n"/>
-      <c r="F112" s="14" t="n"/>
-      <c r="G112" s="14" t="n"/>
-      <c r="H112" s="14" t="n"/>
-    </row>
-    <row r="113">
-      <c r="A113" s="6" t="inlineStr">
-        <is>
-          <t>Carrying value of the very large crude carrier sold (USD 000)</t>
-        </is>
-      </c>
-      <c r="C113" s="27" t="n">
-        <v>83000</v>
-      </c>
-    </row>
-    <row r="114">
-      <c r="A114" s="6" t="inlineStr">
-        <is>
-          <t>Realised sale price, January 2026 (USD 000)</t>
-        </is>
-      </c>
-      <c r="C114" s="27" t="n">
-        <v>111000</v>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" s="6" t="inlineStr">
-        <is>
-          <t>Capital gain recognised on the sale, as disclosed (USD 000)</t>
-        </is>
-      </c>
-      <c r="C115" s="27" t="n">
-        <v>27000</v>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" s="4" t="inlineStr">
+      <c r="A112" s="4" t="inlineStr">
         <is>
           <t>Every figure on this sheet is an input. Nothing here is computed; everything computed from these cells lives on the sheets that follow.</t>
         </is>
@@ -12796,9 +12752,8 @@
           <t>Carrying value of the very large crude carrier sold (USD 000)</t>
         </is>
       </c>
-      <c r="C56" s="18">
-        <f>Assumptions!$C$113</f>
-        <v/>
+      <c r="C56" s="27" t="n">
+        <v>83000</v>
       </c>
     </row>
     <row r="57">
@@ -12807,9 +12762,8 @@
           <t>Realised sale price, January 2026 (USD 000)</t>
         </is>
       </c>
-      <c r="C57" s="18">
-        <f>Assumptions!$C$114</f>
-        <v/>
+      <c r="C57" s="27" t="n">
+        <v>111000</v>
       </c>
     </row>
     <row r="58">
@@ -12829,9 +12783,8 @@
           <t>Capital gain recognised on the sale, as disclosed (USD 000)</t>
         </is>
       </c>
-      <c r="C59" s="18">
-        <f>Assumptions!$C$115</f>
-        <v/>
+      <c r="C59" s="27" t="n">
+        <v>27000</v>
       </c>
     </row>
     <row r="60">

</xml_diff>

<commit_message>
ADNOCLS: second edition — every gate passes on the delivered files
LibreOffice recalculation 0 error cells across 16 sheets; 2,069 of 2,069 formula
cells reproduce the model with 95 headline reconciliations; 85 drivers propagate
in the asserted direction with no dead inputs; 146 row labels each describe their
own row; the documents carry 28 of the model's current figures and none of the
framing this edition replaced.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FX6uP9o59mB1WpgL9CePqV
</commit_message>
<xml_diff>
--- a/engine/adnocls_study/ADNOCLS_Valuation_Model_09082026_public.xlsx
+++ b/engine/adnocls_study/ADNOCLS_Valuation_Model_09082026_public.xlsx
@@ -5101,16 +5101,16 @@
         </is>
       </c>
       <c r="B6" s="21" t="n">
-        <v>8.821143313217801</v>
+        <v>7.684059821165052</v>
       </c>
       <c r="C6" s="21" t="n">
-        <v>9.403767556239309</v>
+        <v>8.089468651542681</v>
       </c>
       <c r="D6" s="21" t="n">
-        <v>10.13964211125459</v>
+        <v>8.585870670520746</v>
       </c>
       <c r="E6" s="21" t="n">
-        <v>11.10110240007209</v>
+        <v>9.209641660332705</v>
       </c>
     </row>
     <row r="7">
@@ -5120,16 +5120,16 @@
         </is>
       </c>
       <c r="B7" s="21" t="n">
-        <v>7.377139043473286</v>
+        <v>6.521904241629056</v>
       </c>
       <c r="C7" s="21" t="n">
-        <v>7.739575354063446</v>
+        <v>6.779643881894967</v>
       </c>
       <c r="D7" s="21" t="n">
-        <v>8.17954270903156</v>
+        <v>7.085238719949822</v>
       </c>
       <c r="E7" s="21" t="n">
-        <v>8.726572606786965</v>
+        <v>7.454596803798754</v>
       </c>
     </row>
     <row r="8">
@@ -5139,16 +5139,16 @@
         </is>
       </c>
       <c r="B8" s="21" t="n">
-        <v>6.336732732190536</v>
+        <v>5.661976211130093</v>
       </c>
       <c r="C8" s="21" t="n">
-        <v>6.573581007511788</v>
+        <v>5.831947183128495</v>
       </c>
       <c r="D8" s="21" t="n">
-        <v>6.852892465948203</v>
+        <v>6.028543766541673</v>
       </c>
       <c r="E8" s="21" t="n">
-        <v>7.188337826923521</v>
+        <v>6.259397237851367</v>
       </c>
     </row>
     <row r="9">
@@ -5158,16 +5158,16 @@
         </is>
       </c>
       <c r="B9" s="21" t="n">
-        <v>5.594985790205619</v>
+        <v>5.036939713504717</v>
       </c>
       <c r="C9" s="21" t="n">
-        <v>5.758498704864779</v>
+        <v>5.154177217420941</v>
       </c>
       <c r="D9" s="21" t="n">
-        <v>5.947214608798108</v>
+        <v>5.287160500641522</v>
       </c>
       <c r="E9" s="21" t="n">
-        <v>6.168263183774388</v>
+        <v>5.439908589636779</v>
       </c>
     </row>
     <row r="10">
@@ -5177,22 +5177,22 @@
         </is>
       </c>
       <c r="B10" s="21" t="n">
-        <v>4.991669767894912</v>
+        <v>4.52102003401324</v>
       </c>
       <c r="C10" s="21" t="n">
-        <v>5.105151875101628</v>
+        <v>4.601537559133286</v>
       </c>
       <c r="D10" s="21" t="n">
-        <v>5.23366042288852</v>
+        <v>4.691207672798638</v>
       </c>
       <c r="E10" s="21" t="n">
-        <v>5.380993860983772</v>
+        <v>4.792139844400095</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>The beta rows are not evenly spaced round numbers. They span the two index constructions and the interval around the adopted one: 0.705 is the equal-weight composite of the exchange's own names, 1.085 is the adopted regression against the exchange's published index, and 1.412 is the top of that regression's own 90% confidence interval (its bottom, 0.758, sits just above the composite reading). READ THIS GRID AS A SHAPE, NOT AS A LEVEL. Every cell is a complete re-run of the model discounted at a rate built from the equity and the debt alone. The rate the valuation itself uses also carries the perpetual capital securities at their own coupon, which makes it dearer — 8.49% against 7.86% over the forecast years and 7.73% against 7.16% in the terminal — so every cell here sits above the published figure. At the 1.085 row and the 2.0% column the grid reads AED 6.85 against the published AED 6.03, a gap of 13.7%. What the grid is for is the slope: how much the answer moves for a given move in the beta or in terminal growth.</t>
+          <t>The beta rows are not evenly spaced round numbers. They span the two index constructions and the interval around the adopted one: 0.705 is the equal-weight composite of the exchange's own names, 1.085 is the adopted regression against the exchange's published index, and 1.412 is the top of that regression's own 90% confidence interval (its bottom, 0.758, sits just above the composite reading). The terminal growth column at 2.0% is the one the model runs on, so the cell where that column meets the 1.085 row is the published cash-flow value of AED 6.03 — every cell here is a complete re-run of the model discounted at the same three tranches of capital the valuation itself uses, equity, debt and the perpetual securities, so the grid is centred on the figure it brackets.</t>
         </is>
       </c>
     </row>
@@ -5245,19 +5245,19 @@
         </is>
       </c>
       <c r="B14" s="21" t="n">
-        <v>5.185674797723733</v>
+        <v>5.121306811301282</v>
       </c>
       <c r="C14" s="21" t="n">
-        <v>5.644016771814515</v>
+        <v>5.574925288921477</v>
       </c>
       <c r="D14" s="21" t="n">
-        <v>6.102358745905295</v>
+        <v>6.028543766541673</v>
       </c>
       <c r="E14" s="21" t="n">
-        <v>6.560700719996079</v>
+        <v>6.482162244161869</v>
       </c>
       <c r="F14" s="21" t="n">
-        <v>7.019042694086861</v>
+        <v>6.935780721782064</v>
       </c>
     </row>
     <row r="15">
@@ -5274,7 +5274,7 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>The same caution applies to this row and the one below it: each is a re-run discounted over the forecast years at 7.86%, the rate the equity and the debt alone imply, rather than at the 8.49% the valuation uses. At 1.00x it reads AED 6.10 against the published AED 6.03, 1.2% above it. The swing across the row is what it is for.</t>
+          <t>This row and the one below it are re-runs of the whole model at the same 8.49% cost of capital the valuation uses, so the 1.00x cell reproduces the published AED 6.03 exactly and the swing across the row is a clean read of what that single driver is worth.</t>
         </is>
       </c>
     </row>
@@ -5322,16 +5322,16 @@
         </is>
       </c>
       <c r="B19" s="21" t="n">
-        <v>6.515320858093369</v>
+        <v>6.437907235122407</v>
       </c>
       <c r="C19" s="21" t="n">
-        <v>6.102358745905295</v>
+        <v>6.028543766541673</v>
       </c>
       <c r="D19" s="21" t="n">
-        <v>5.689396633717223</v>
+        <v>5.619180297960939</v>
       </c>
       <c r="E19" s="21" t="n">
-        <v>5.276434521529151</v>
+        <v>5.209816829380204</v>
       </c>
     </row>
     <row r="20">
@@ -7557,7 +7557,7 @@
         </is>
       </c>
       <c r="C6" s="21" t="n">
-        <v>3.840998691014435</v>
+        <v>3.790471085198643</v>
       </c>
     </row>
     <row r="7" ht="28" customHeight="1">
@@ -7572,7 +7572,7 @@
         </is>
       </c>
       <c r="C7" s="21" t="n">
-        <v>9.379477215384453</v>
+        <v>9.270835477800441</v>
       </c>
     </row>
     <row r="8" ht="28" customHeight="1">
@@ -18332,11 +18332,11 @@
     <row r="117">
       <c r="A117" s="6" t="inlineStr">
         <is>
-          <t>Cost of capital — explicit window, composite-index beta. The contested change is the cost of EQUITY, so the alternative reprices the equity leg over the explicit window and leaves the perpetual leg to the terminal, where its cost has normalised</t>
+          <t>Cost of capital — explicit window, composite-index beta. Only the cost of EQUITY changes: the same three tranches of capital are carried, because how the market is measured does not change what the company is financed with</t>
         </is>
       </c>
       <c r="C117" s="49">
-        <f>C101*C115+C102*C94</f>
+        <f>C101*C115+C102*C94+C103*C104</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
ADNOCLS: final delivered artefacts, all gates green
The workbook rebuild landed after the previous commit, so the delivered files are
refreshed here against it. Every gate re-run on these exact files: LibreOffice 0
error cells, 2,069 of 2,069 formula cells reproducing the model, 85 drivers
propagating, 146 labels correct, documents current, scrub clean.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FX6uP9o59mB1WpgL9CePqV
</commit_message>
<xml_diff>
--- a/engine/adnocls_study/ADNOCLS_Valuation_Model_09082026_public.xlsx
+++ b/engine/adnocls_study/ADNOCLS_Valuation_Model_09082026_public.xlsx
@@ -544,7 +544,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I66"/>
+  <dimension ref="A1:I93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="114" customWidth="1" min="1" max="1"/>
@@ -683,307 +683,488 @@
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>THREE THINGS ARE PASTED VALUES, and it is worth knowing exactly which.</t>
+          <t>FOUR THINGS ARE PASTED VALUES, and it is worth knowing exactly which.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  (1) AUDITED AND DISCLOSED HISTORY — the primary record, not a calculation. Where a line is both disclosed</t>
+          <t xml:space="preserve">  (1) THE INDEPENDENT INPUTS ON THE ASSUMPTIONS SHEET — the blue cells: disclosed vessel counts, published</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">      and arithmetically derivable, the DISCLOSED figure is carried, because the filing is the record.</t>
+          <t xml:space="preserve">      day rates, the twelve charter fixtures and their dates, the balance-sheet anchors, the tax rates and</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  (2) THE OUTPUT OF A UNIT BUILD that would be unreadable flattened into a grid — the historical segment</t>
+          <t xml:space="preserve">      the study judgements. Anything on that sheet that is itself DERIVED from other inputs is a GREEN</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">      revenue and earnings table, which the operating-segments note gives directly.</t>
+          <t xml:space="preserve">      formula pointing at the build that produces it — the running cost per vessel-day, the gas-carrier day</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  (3) WHOLE-MODEL RE-RUNS, where each figure is a complete revaluation of the entire model and so cannot be</t>
+          <t xml:space="preserve">      rate, the three days ratios and the opening working capital are all solved elsewhere and only shown</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">      a single formula: the Monte Carlo price map, the two sensitivity grids, the discounted-cash-flow</t>
+          <t xml:space="preserve">      there, so a reader can never mistake an output for an assumption.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">      bear and bull bounds (each of which re-runs the fleet build at a different rate anchor, a different</t>
+          <t xml:space="preserve">  (2) AUDITED AND DISCLOSED HISTORY — the primary record, not a calculation. Where a line is both disclosed</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">      beta — the two ends of the regression's own confidence interval — and a different capital-expenditure</t>
+          <t xml:space="preserve">      and arithmetically derivable, the DISCLOSED figure is carried, because the filing is the record.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">      path) and the three expert-panel legs.</t>
+          <t xml:space="preserve">  (3) THE OUTPUT OF A UNIT BUILD that would be unreadable flattened into a grid — the historical segment</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  THE MONTE CARLO AND SENSITIVITY GRIDS DO NOT REDRAW WHEN A DRIVER IS CHANGED. Changing a blue cell</t>
+          <t xml:space="preserve">      revenue and earnings table, which the operating-segments note gives directly.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  reprices the whole valuation chain, but those grids are engine outputs and stay as they were run.</t>
+          <t xml:space="preserve">  (4) WHOLE-MODEL RE-RUNS, where each figure is a complete revaluation of the entire model and so cannot be</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Anything else pasted is a defect.</t>
+          <t xml:space="preserve">      a single formula: the Monte Carlo price map, the two sensitivity grids, the discounted-cash-flow</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="3" t="inlineStr"/>
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      bear and bull bounds (each of which re-runs the fleet build at a different rate anchor, a different</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>How revenue is built. Not as one growth rate. The tanker fleet is built vessel by vessel: fifty-three owned</t>
+          <t xml:space="preserve">      beta — the two ends of the regression's own confidence interval — and a different capital-expenditure</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>vessels split into those trading at spot rates and those on charters out at rates already fixed and</t>
+          <t xml:space="preserve">      path) and the three expert-panel legs.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>disclosed, each class earning its own time-charter equivalent per day over 365 days, less an all-in running</t>
+          <t xml:space="preserve">  THE MONTE CARLO AND SENSITIVITY GRIDS DO NOT REDRAW WHEN A DRIVER IS CHANGED. Changing a blue cell</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>cost per vessel per day escalated on a services-and-wage escalator. The gas carriers are built from</t>
+          <t xml:space="preserve">  reprices the whole valuation chain, but those grids are engine outputs and stay as they were run.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>contracted vessel-years times an implied day rate. The five remaining units are grown on their own revenue</t>
+          <t xml:space="preserve">  Anything else pasted is a defect.</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="3" t="inlineStr">
-        <is>
-          <t>and margin drivers, anchored on what each actually earned in the first quarter of 2026.</t>
-        </is>
-      </c>
+      <c r="A39" s="3" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" s="3" t="inlineStr"/>
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>How revenue is built. Not as one growth rate, and not off the published rate either. The company gives one</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>THE CONTESTED JUDGEMENT, PUBLISHED BOTH WAYS — HOW THE MARKET IS MEASURED. The same weekly regression of the</t>
+          <t>rate per vessel class each quarter, and its own chief financial officer said on the first-quarter call that</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>stock's own returns is run against two different measures of its market, and the answer moves a long way</t>
+          <t>this rate is a BLEND across the whole class, the vessels on charters out included. So the SPOT rate is not</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>between them. Against the published index of the exchange the share is listed on — the index the method</t>
+          <t>read off that disclosure — it is SOLVED out of it, window by window: the published blend times the class</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>asks for, and the primary reading — the beta is 1.085. Against an equal-weight composite of that same</t>
+          <t>vessel-days, less the revenue the twelve disclosed fixtures earn over exactly the days their own contracts</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>exchange's names, which gives its smallest listings the same say as its largest, the beta is</t>
+          <t>run, divided by the vessel-days that actually traded spot. Every step of that derivation is on the Segments</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>0.705. The published index is weighted by size and is therefore dominated by the very group this</t>
+          <t>sheet, cell by cell. The forecast then prices each vessel on its own terms — chartered vessels at their</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>company belongs to; the composite is not. That single difference in construction, and nothing about the</t>
+          <t>contracted rate for their contracted days, everything else at the implied spot rate — less an all-in running</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
         <is>
-          <t>company, moves the cost of equity and the cash-flow value materially. BOTH are carried through the model in</t>
+          <t>cost per vessel-day that is itself solved so the same construction reproduces the tanker earnings the company</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>full, side by side, on the Summary, Fundamental Valuation and DCF sheets. They are NOT averaged into one</t>
+          <t>reported for 2025. The gas carriers are contracted vessel-years times a day rate solved the same way. The</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>number. The regression's own 90% confidence interval on the primary estimate runs 0.758 to 1.412, and</t>
+          <t>five remaining units are grown on their own revenue and margin drivers, anchored on what each actually</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>those two bounds — not round numbers chosen by hand — are the betas used in the bear and bull cases, so the</t>
+          <t>earned in the first quarter of 2026.</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="3" t="inlineStr">
-        <is>
-          <t>published range is the range the estimate itself supports.</t>
-        </is>
-      </c>
+      <c r="A52" s="3" t="inlineStr"/>
     </row>
     <row r="53">
-      <c r="A53" s="3" t="inlineStr"/>
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>THE COST OF CAPITAL CARRIES THREE TRANCHES, NOT TWO: equity, debt, and the perpetual capital securities at</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>What it is not. It is not investment advice, a recommendation, or a price target. Values are model outputs</t>
+          <t>their own coupon. Those securities rank ahead of the ordinary shares and are deducted in the equity bridge,</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>shown as ranges and distributions.</t>
+          <t>and a claim that is deducted from enterprise value has to be weighted in the rate as well — the two are</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="3" t="inlineStr"/>
+      <c r="A56" s="3" t="inlineStr">
+        <is>
+          <t>halves of one treatment. The coupon is an equity distribution rather than interest, so it is not taxed down.</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>Sourcing note, up front. FY2023, FY2024 and FY2025 come from the company's own audited consolidated</t>
+          <t>Every construction in the workbook carries the same three tranches, including the sensitivity re-runs, so</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
         <is>
-          <t>financial statements; the first quarter of 2026 comes from the reviewed interim statements; the fleet,</t>
+          <t>the sensitivity grid is centred on the figure it brackets.</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="3" t="inlineStr">
-        <is>
-          <t>rate and contract data come from the company's own investor presentations and earnings calls. Every input</t>
-        </is>
-      </c>
+      <c r="A59" s="3" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>is listed with its value, source and date in the companion bibliography document.</t>
+          <t>THE BOOK LENS IS A RESIDUAL INCOME BUILD. A single-stage justified price-to-book assumes a steady state this</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="3" t="inlineStr"/>
+      <c r="A61" s="3" t="inlineStr">
+        <is>
+          <t>company is not in: it pays out about a third of its earnings and compounds its book above its own cost of</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
         <is>
-          <t>Currency. US dollar thousand unless stated — the company reports in US dollars. Per-share figures are in</t>
+          <t>equity, where that formula is undefined rather than merely wrong. The lens is instead the book the company</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>dirhams at the fixed parity of 3.6725 dirhams to the dollar. Spot AED 6.16 (2026-08-07 close).</t>
+          <t>already has, plus the present value of earning more than the cost of equity on it for five years, plus a</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="3" t="inlineStr">
         <is>
-          <t>Sheets: READ FIRST · Summary · Fundamental Valuation · Assumptions · SOTP Bridge · Segments · Relative &amp;</t>
+          <t>remainder in which that excess fades. The whole ladder is live on the Relative &amp; Normalized sheet, three</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>Normalized · DCF · Income Statement · Balance Sheet · Cash Flow · Summary Financials · Monte Carlo ·</t>
+          <t>times over — base, bear and bull — and the return it is struck on is what the ORDINARY holders earn, after</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="3" t="inlineStr">
+        <is>
+          <t>the perpetual coupon that ranks ahead of them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="3" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="3" t="inlineStr">
+        <is>
+          <t>THE CONTESTED JUDGEMENT, PUBLISHED BOTH WAYS — HOW THE MARKET IS MEASURED. The same weekly regression of the</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="3" t="inlineStr">
+        <is>
+          <t>stock's own returns is run against two different measures of its market, and the answer moves a long way</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="3" t="inlineStr">
+        <is>
+          <t>between them. Against the published index of the exchange the share is listed on — the index the method</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="3" t="inlineStr">
+        <is>
+          <t>asks for, and the primary reading — the beta is 1.085. Against an equal-weight composite of that same</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="3" t="inlineStr">
+        <is>
+          <t>exchange's names, which gives its smallest listings the same say as its largest, the beta is</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="3" t="inlineStr">
+        <is>
+          <t>0.705. The published index is weighted by size and is therefore dominated by the very group this</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="3" t="inlineStr">
+        <is>
+          <t>company belongs to; the composite is not. That single difference in construction, and nothing about the</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="3" t="inlineStr">
+        <is>
+          <t>company, moves the cost of equity and the cash-flow value materially. BOTH are carried through the model in</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="3" t="inlineStr">
+        <is>
+          <t>full, side by side, on the Summary, Fundamental Valuation and DCF sheets. They are NOT averaged into one</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="3" t="inlineStr">
+        <is>
+          <t>number. The regression's own 90% confidence interval on the primary estimate runs 0.758 to 1.412, and</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="3" t="inlineStr">
+        <is>
+          <t>those two bounds — not round numbers chosen by hand — are the betas used in the bear and bull cases, so the</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="3" t="inlineStr">
+        <is>
+          <t>published range is the range the estimate itself supports.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="3" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="3" t="inlineStr">
+        <is>
+          <t>What it is not. It is not investment advice, a recommendation, or a price target. Values are model outputs</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="3" t="inlineStr">
+        <is>
+          <t>shown as ranges and distributions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="3" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="3" t="inlineStr">
+        <is>
+          <t>Sourcing note, up front. FY2023, FY2024 and FY2025 come from the company's own audited consolidated</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="3" t="inlineStr">
+        <is>
+          <t>financial statements; the first quarter of 2026 comes from the reviewed interim statements; the fleet,</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="3" t="inlineStr">
+        <is>
+          <t>rate and contract data come from the company's own investor presentations and earnings calls. Every input</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="3" t="inlineStr">
+        <is>
+          <t>is listed with its value, source and date in the companion bibliography document.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="3" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="3" t="inlineStr">
+        <is>
+          <t>Currency. US dollar thousand unless stated — the company reports in US dollars. Per-share figures are in</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="3" t="inlineStr">
+        <is>
+          <t>dirhams at the fixed parity of 3.6725 dirhams to the dollar. Spot AED 6.16 (2026-08-07 close).</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="3" t="inlineStr">
+        <is>
+          <t>Sheets: READ FIRST · Summary · Fundamental Valuation · Assumptions · SOTP Bridge · Segments · Relative &amp;</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="3" t="inlineStr">
+        <is>
+          <t>Normalized · DCF · Income Statement · Balance Sheet · Cash Flow · Summary Financials · Monte Carlo ·</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="3" t="inlineStr">
         <is>
           <t>Sensitivity · Per-Share &amp; Ratios · Peer &amp; Sector.</t>
         </is>
@@ -7615,7 +7796,7 @@
       </c>
       <c r="B10" s="20" t="inlineStr">
         <is>
-          <t>justified price-to-book on the sustainable return on equity</t>
+          <t>the book the company already has, plus the present value of earning more than the cost of equity on it while that lasts, plus a fading remainder — a residual income build, not a justified multiple</t>
         </is>
       </c>
       <c r="C10" s="7">

</xml_diff>

<commit_message>
ADNOCLS: deliverables mid-rebuild on the sanctioned beta
Committed so the tree is clean while the study, workbook and bibliography finish
re-rendering. The copies under files/ still carry the pre-re-derivation beta and
are deliberately NOT shipped until they match the page.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FX6uP9o59mB1WpgL9CePqV
</commit_message>
<xml_diff>
--- a/engine/adnocls_study/ADNOCLS_Valuation_Model_09082026_public.xlsx
+++ b/engine/adnocls_study/ADNOCLS_Valuation_Model_09082026_public.xlsx
@@ -545,7 +545,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I115"/>
+  <dimension ref="A1:I126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="114" customWidth="1" min="1" max="1"/>
@@ -970,352 +970,425 @@
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
         <is>
-          <t>How revenue is built. Not as one growth rate, and not off the published rate either. The company gives one</t>
+          <t>AND THE BETA HAS BEEN RE-MEASURED. It is now produced by the same standard routine used for every share</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>rate per vessel class each quarter, and its own chief financial officer said on the first-quarter call that</t>
+          <t>covered on this desk: the market series is resolved from the exchange the share is listed on rather than</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="3" t="inlineStr">
         <is>
-          <t>this rate is a BLEND across the whole class, the vessels on charters out included. So the SPOT rate is not</t>
+          <t>chosen, both series are screened for data quality before they are paired, and the weekly returns are</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>read off that disclosure — it is SOLVED out of it, window by window: the published blend times the class</t>
+          <t>measured on that exchange's own trading week. The series it resolved is the one this study already used, so</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="3" t="inlineStr">
         <is>
-          <t>vessel-days, less the revenue the twelve disclosed fixtures earn over exactly the days their own contracts</t>
+          <t>WHICH market the share is measured against has not changed — but the grid and the screening do move the</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>run, divided by the vessel-days that actually traded spot. Every step of that derivation is on the Segments</t>
+          <t>figure: the slope is now 1.1032 on 159 weekly observations, and its 90% confidence interval</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="3" t="inlineStr">
         <is>
-          <t>sheet, cell by cell. The forecast then prices each vessel on its own terms — chartered vessels at their</t>
+          <t>runs 0.586 to 1.621, materially WIDER than the interval the previous edition</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>contracted rate for their contracted days, everything else at the implied spot rate — less an all-in running</t>
+          <t>published. The bear and bull cases take those two bounds directly, so the published range widens with it.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="3" t="inlineStr">
         <is>
-          <t>cost per vessel-day that is itself solved so the same construction reproduces the tanker earnings the company</t>
+          <t>A range that widens on re-measurement is information about how much a three-year price history can settle,</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
         <is>
-          <t>reported for 2025. The gas carriers are contracted vessel-years times a day rate solved the same way. The</t>
+          <t>not an embarrassment to be smoothed away.</t>
         </is>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="3" t="inlineStr">
-        <is>
-          <t>five remaining units are grown on their own revenue and margin drivers, anchored on what each actually</t>
-        </is>
-      </c>
+      <c r="A72" s="3" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="3" t="inlineStr">
         <is>
-          <t>earned in the first quarter of 2026.</t>
+          <t>How revenue is built. Not as one growth rate, and not off the published rate either. The company gives one</t>
         </is>
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="3" t="inlineStr"/>
+      <c r="A74" s="3" t="inlineStr">
+        <is>
+          <t>rate per vessel class each quarter, and its own chief financial officer said on the first-quarter call that</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
         <is>
-          <t>THE COST OF CAPITAL CARRIES THREE TRANCHES, NOT TWO: equity, debt, and the perpetual capital securities at</t>
+          <t>this rate is a BLEND across the whole class, the vessels on charters out included. So the SPOT rate is not</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="3" t="inlineStr">
         <is>
-          <t>their own coupon. Those securities rank ahead of the ordinary shares and are deducted in the equity bridge,</t>
+          <t>read off that disclosure — it is SOLVED out of it, window by window: the published blend times the class</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
         <is>
-          <t>and a claim that is deducted from enterprise value has to be weighted in the rate as well — the two are</t>
+          <t>vessel-days, less the revenue the twelve disclosed fixtures earn over exactly the days their own contracts</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="3" t="inlineStr">
         <is>
-          <t>halves of one treatment. The coupon is an equity distribution rather than interest, so it is not taxed down.</t>
+          <t>run, divided by the vessel-days that actually traded spot. Every step of that derivation is on the Segments</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="3" t="inlineStr">
         <is>
-          <t>Every construction in the workbook carries the same three tranches, including the sensitivity re-runs, so</t>
+          <t>sheet, cell by cell. The forecast then prices each vessel on its own terms — chartered vessels at their</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="3" t="inlineStr">
         <is>
-          <t>the sensitivity grid is centred on the figure it brackets.</t>
+          <t>contracted rate for their contracted days, everything else at the implied spot rate — less an all-in running</t>
         </is>
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="3" t="inlineStr"/>
+      <c r="A81" s="3" t="inlineStr">
+        <is>
+          <t>cost per vessel-day that is itself solved so the same construction reproduces the tanker earnings the company</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="3" t="inlineStr">
         <is>
-          <t>THE BOOK LENS IS A RESIDUAL INCOME BUILD. A single-stage justified price-to-book assumes a steady state this</t>
+          <t>reported for 2025. The gas carriers are contracted vessel-years times a day rate solved the same way. The</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="3" t="inlineStr">
         <is>
-          <t>company is not in: it pays out about a third of its earnings and compounds its book above its own cost of</t>
+          <t>five remaining units are grown on their own revenue and margin drivers, anchored on what each actually</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="3" t="inlineStr">
         <is>
-          <t>equity, where that formula is undefined rather than merely wrong. The lens is instead the book the company</t>
+          <t>earned in the first quarter of 2026.</t>
         </is>
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="3" t="inlineStr">
-        <is>
-          <t>already has, plus the present value of earning more than the cost of equity on it for five years, plus a</t>
-        </is>
-      </c>
+      <c r="A85" s="3" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="3" t="inlineStr">
         <is>
-          <t>remainder in which that excess fades. The whole ladder is live on the Relative &amp; Normalized sheet, three</t>
+          <t>THE COST OF CAPITAL CARRIES THREE TRANCHES, NOT TWO: equity, debt, and the perpetual capital securities at</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="3" t="inlineStr">
         <is>
-          <t>times over — base, bear and bull — and the return it is struck on is what the ORDINARY holders earn, after</t>
+          <t>their own coupon. Those securities rank ahead of the ordinary shares and are deducted in the equity bridge,</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="3" t="inlineStr">
         <is>
-          <t>the perpetual coupon that ranks ahead of them.</t>
+          <t>and a claim that is deducted from enterprise value has to be weighted in the rate as well — the two are</t>
         </is>
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="3" t="inlineStr"/>
+      <c r="A89" s="3" t="inlineStr">
+        <is>
+          <t>halves of one treatment. The coupon is an equity distribution rather than interest, so it is not taxed down.</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="3" t="inlineStr">
         <is>
-          <t>THE CONTESTED JUDGEMENT, PUBLISHED BOTH WAYS — HOW THE MARKET IS MEASURED. The same weekly regression of the</t>
+          <t>Every construction in the workbook carries the same three tranches, including the sensitivity re-runs, so</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="3" t="inlineStr">
         <is>
-          <t>stock's own returns is run against two different measures of its market, and the answer moves a long way</t>
+          <t>the sensitivity grid is centred on the figure it brackets.</t>
         </is>
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="3" t="inlineStr">
-        <is>
-          <t>between them. Against the published index of the exchange the share is listed on — the index the method</t>
-        </is>
-      </c>
+      <c r="A92" s="3" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" s="3" t="inlineStr">
         <is>
-          <t>asks for, and the primary reading — the beta is 1.085. Against an equal-weight composite of that same</t>
+          <t>THE BOOK LENS IS A RESIDUAL INCOME BUILD. A single-stage justified price-to-book assumes a steady state this</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="3" t="inlineStr">
         <is>
-          <t>exchange's names, which gives its smallest listings the same say as its largest, the beta is</t>
+          <t>company is not in: it pays out about a third of its earnings and compounds its book above its own cost of</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="3" t="inlineStr">
         <is>
-          <t>0.705. The published index is weighted by size and is therefore dominated by the very group this</t>
+          <t>equity, where that formula is undefined rather than merely wrong. The lens is instead the book the company</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="3" t="inlineStr">
         <is>
-          <t>company belongs to; the composite is not. That single difference in construction, and nothing about the</t>
+          <t>already has, plus the present value of earning more than the cost of equity on it for five years, plus a</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="3" t="inlineStr">
         <is>
-          <t>company, moves the cost of equity and the cash-flow value materially. BOTH are carried through the model in</t>
+          <t>remainder in which that excess fades. The whole ladder is live on the Relative &amp; Normalized sheet, three</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="3" t="inlineStr">
         <is>
-          <t>full, side by side, on the Summary, Fundamental Valuation and DCF sheets. They are NOT averaged into one</t>
+          <t>times over — base, bear and bull — and the return it is struck on is what the ORDINARY holders earn, after</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="3" t="inlineStr">
         <is>
-          <t>number. The regression's own 90% confidence interval on the primary estimate runs 0.758 to 1.412, and</t>
+          <t>the perpetual coupon that ranks ahead of them.</t>
         </is>
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="3" t="inlineStr">
-        <is>
-          <t>those two bounds — not round numbers chosen by hand — are the betas used in the bear and bull cases, so the</t>
-        </is>
-      </c>
+      <c r="A100" s="3" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="3" t="inlineStr">
         <is>
-          <t>published range is the range the estimate itself supports.</t>
+          <t>THE CONTESTED JUDGEMENT, PUBLISHED BOTH WAYS — HOW THE MARKET IS MEASURED. The same weekly regression of the</t>
         </is>
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="3" t="inlineStr"/>
+      <c r="A102" s="3" t="inlineStr">
+        <is>
+          <t>stock's own returns is run against two different measures of its market, and the answer moves a long way</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="3" t="inlineStr">
         <is>
-          <t>What it is not. It is not investment advice, a recommendation, or a price target. Values are model outputs</t>
+          <t>between them. Against the published index of the exchange the share is listed on — the index the method</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="3" t="inlineStr">
         <is>
-          <t>shown as ranges and distributions.</t>
+          <t>asks for, and the primary reading — the beta is 1.103. Against an equal-weight composite of that same</t>
         </is>
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="3" t="inlineStr"/>
+      <c r="A105" s="3" t="inlineStr">
+        <is>
+          <t>exchange's names, which gives its smallest listings the same say as its largest, the beta is</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="3" t="inlineStr">
         <is>
-          <t>Sourcing note, up front. FY2023, FY2024 and FY2025 come from the company's own audited consolidated</t>
+          <t>0.705. The published index is weighted by size and is therefore dominated by the very group this</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="3" t="inlineStr">
         <is>
-          <t>financial statements; the first quarter of 2026 comes from the reviewed interim statements; the fleet,</t>
+          <t>company belongs to; the composite is not. That single difference in construction, and nothing about the</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="3" t="inlineStr">
         <is>
-          <t>rate and contract data come from the company's own investor presentations and earnings calls. Every input</t>
+          <t>company, moves the cost of equity and the cash-flow value materially. BOTH are carried through the model in</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="3" t="inlineStr">
         <is>
-          <t>is listed with its value, source and date in the companion bibliography document.</t>
+          <t>full, side by side, on the Summary, Fundamental Valuation and DCF sheets. They are NOT averaged into one</t>
         </is>
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="3" t="inlineStr"/>
+      <c r="A110" s="3" t="inlineStr">
+        <is>
+          <t>number. The regression's own 90% confidence interval on the primary estimate runs 0.586 to 1.621, and</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="3" t="inlineStr">
         <is>
-          <t>Currency. US dollar thousand unless stated — the company reports in US dollars. Per-share figures are in</t>
+          <t>those two bounds — not round numbers chosen by hand — are the betas used in the bear and bull cases, so the</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="3" t="inlineStr">
         <is>
-          <t>dirhams at the fixed parity of 3.6725 dirhams to the dollar. Spot AED 6.16 (2026-08-07 close).</t>
+          <t>published range is the range the estimate itself supports.</t>
         </is>
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="3" t="inlineStr">
-        <is>
-          <t>Sheets: READ FIRST · Summary · Fundamental Valuation · Assumptions · SOTP Bridge · Segments · Relative &amp;</t>
-        </is>
-      </c>
+      <c r="A113" s="3" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" s="3" t="inlineStr">
         <is>
-          <t>Normalized · DCF · Income Statement · Balance Sheet · Cash Flow · Summary Financials · Monte Carlo ·</t>
+          <t>What it is not. It is not investment advice, a recommendation, or a price target. Values are model outputs</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="3" t="inlineStr">
+        <is>
+          <t>shown as ranges and distributions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="3" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="3" t="inlineStr">
+        <is>
+          <t>Sourcing note, up front. FY2023, FY2024 and FY2025 come from the company's own audited consolidated</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="3" t="inlineStr">
+        <is>
+          <t>financial statements; the first quarter of 2026 comes from the reviewed interim statements; the fleet,</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="3" t="inlineStr">
+        <is>
+          <t>rate and contract data come from the company's own investor presentations and earnings calls. Every input</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="3" t="inlineStr">
+        <is>
+          <t>is listed with its value, source and date in the companion bibliography document.</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="3" t="inlineStr"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="3" t="inlineStr">
+        <is>
+          <t>Currency. US dollar thousand unless stated — the company reports in US dollars. Per-share figures are in</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="3" t="inlineStr">
+        <is>
+          <t>dirhams at the fixed parity of 3.6725 dirhams to the dollar. Spot AED 6.16 (2026-08-07 close).</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="3" t="inlineStr">
+        <is>
+          <t>Sheets: READ FIRST · Summary · Fundamental Valuation · Assumptions · SOTP Bridge · Segments · Relative &amp;</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="3" t="inlineStr">
+        <is>
+          <t>Normalized · DCF · Income Statement · Balance Sheet · Cash Flow · Summary Financials · Monte Carlo ·</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="3" t="inlineStr">
         <is>
           <t>Sensitivity · Per-Share &amp; Ratios · Peer &amp; Sector.</t>
         </is>
@@ -5497,64 +5570,64 @@
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>1.085</t>
+          <t>1.103</t>
         </is>
       </c>
       <c r="B8" s="21" t="n">
-        <v>6.104211768824626</v>
+        <v>6.020153084134909</v>
       </c>
       <c r="C8" s="21" t="n">
-        <v>6.290365806735382</v>
+        <v>6.198777837752638</v>
       </c>
       <c r="D8" s="21" t="n">
-        <v>6.50557697172203</v>
+        <v>6.404817896532908</v>
       </c>
       <c r="E8" s="21" t="n">
-        <v>6.758173447014873</v>
+        <v>6.646025779733348</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>1.250</t>
+          <t>1.350</t>
         </is>
       </c>
       <c r="B9" s="21" t="n">
-        <v>5.400935220772635</v>
+        <v>5.031072269544037</v>
       </c>
       <c r="C9" s="21" t="n">
-        <v>5.528638734441224</v>
+        <v>5.132117653317763</v>
       </c>
       <c r="D9" s="21" t="n">
-        <v>5.673387508676271</v>
+        <v>5.245334010186813</v>
       </c>
       <c r="E9" s="21" t="n">
-        <v>5.839532255632811</v>
+        <v>5.373634668456338</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>1.412</t>
+          <t>1.621</t>
         </is>
       </c>
       <c r="B10" s="21" t="n">
-        <v>4.819724922415764</v>
+        <v>4.192019140583034</v>
       </c>
       <c r="C10" s="21" t="n">
-        <v>4.906776041409081</v>
+        <v>4.242712935566582</v>
       </c>
       <c r="D10" s="21" t="n">
-        <v>5.003609464167625</v>
+        <v>4.297604675716044</v>
       </c>
       <c r="E10" s="21" t="n">
-        <v>5.112479795523905</v>
+        <v>4.357554251269803</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>The beta rows are not evenly spaced round numbers. They span the two index constructions and the interval around the adopted one: 0.705 is the equal-weight composite of the exchange's own names, 1.085 is the adopted regression against the exchange's published index, and 1.412 is the top of that regression's own 90% confidence interval (its bottom, 0.758, sits just above the composite reading). The terminal growth column at 2.0% is the one the model runs on, so the cell where that column meets the 1.085 row is the published cash-flow value of AED 6.51 — every cell here is a complete re-run of the model discounted at the same three tranches of capital the valuation itself uses, equity, debt and the perpetual securities, so the grid is centred on the figure it brackets.</t>
+          <t>The beta rows are not evenly spaced round numbers. They span the two index constructions and the interval around the adopted one: 0.705 is the equal-weight composite of the exchange's own names, 1.103 is the adopted regression against the exchange's published index, and 1.621 is the top of that regression's own 90% confidence interval (its bottom, 0.586, sits below the composite reading, so the bull case is struck outside this grid). The terminal growth column at 2.0% is the one the model runs on, so the cell where that column meets the 1.103 row is the published cash-flow value of AED 6.40 — every cell here is a complete re-run of the model discounted at the same three tranches of capital the valuation itself uses, equity, debt and the perpetual securities, so the grid is centred on the figure it brackets.</t>
         </is>
       </c>
     </row>
@@ -5607,19 +5680,19 @@
         </is>
       </c>
       <c r="B14" s="21" t="n">
-        <v>5.466895404238599</v>
+        <v>5.380506785289913</v>
       </c>
       <c r="C14" s="21" t="n">
-        <v>5.986236187980316</v>
+        <v>5.892662340911411</v>
       </c>
       <c r="D14" s="21" t="n">
-        <v>6.50557697172203</v>
+        <v>6.404817896532908</v>
       </c>
       <c r="E14" s="21" t="n">
-        <v>7.024917755463745</v>
+        <v>6.916973452154407</v>
       </c>
       <c r="F14" s="21" t="n">
-        <v>7.544258539205458</v>
+        <v>7.429129007775901</v>
       </c>
     </row>
     <row r="15">
@@ -5636,7 +5709,7 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>This row and the one below it are re-runs of the whole model at the same 8.49% cost of capital the valuation uses, so the 1.00x cell reproduces the published AED 6.51 exactly and the swing across the row is a clean read of what that single driver is worth.</t>
+          <t>This row and the one below it are re-runs of the whole model at the same 8.56% cost of capital the valuation uses, so the 1.00x cell reproduces the published AED 6.40 exactly and the swing across the row is a clean read of what that single driver is worth.</t>
         </is>
       </c>
     </row>
@@ -5684,16 +5757,16 @@
         </is>
       </c>
       <c r="B19" s="21" t="n">
-        <v>6.914940440302763</v>
+        <v>6.81087218594573</v>
       </c>
       <c r="C19" s="21" t="n">
-        <v>6.50557697172203</v>
+        <v>6.404817896532908</v>
       </c>
       <c r="D19" s="21" t="n">
-        <v>6.096213503141294</v>
+        <v>5.998763607120084</v>
       </c>
       <c r="E19" s="21" t="n">
-        <v>5.686850034560557</v>
+        <v>5.592709317707262</v>
       </c>
     </row>
     <row r="20">
@@ -5746,13 +5819,13 @@
         </is>
       </c>
       <c r="B24" s="21" t="n">
-        <v>6.415224723153202</v>
+        <v>6.315163657148892</v>
       </c>
       <c r="C24" s="21" t="n">
-        <v>5.963130365206823</v>
+        <v>5.868212089093989</v>
       </c>
       <c r="D24" s="21" t="n">
-        <v>5.284988828287254</v>
+        <v>5.197784737011633</v>
       </c>
     </row>
     <row r="25">
@@ -7981,11 +8054,11 @@
       </c>
       <c r="B6" s="20" t="inlineStr">
         <is>
-          <t>beta 1.412 — the TOP of the regression's own 90% confidence interval, not a round number picked by hand — with the rate anchor at 0.85x and capital expenditure at 1.10x. A whole-model re-run</t>
+          <t>beta 1.621 — the TOP of the regression's own 90% confidence interval, not a round number picked by hand — with the rate anchor at 0.85x and capital expenditure at 1.10x. A whole-model re-run</t>
         </is>
       </c>
       <c r="C6" s="21" t="n">
-        <v>4.025007328525061</v>
+        <v>3.417404968021705</v>
       </c>
     </row>
     <row r="7" ht="28" customHeight="1">
@@ -7996,11 +8069,11 @@
       </c>
       <c r="B7" s="20" t="inlineStr">
         <is>
-          <t>beta 0.758 — the BOTTOM of the same interval — with the rate anchor at 1.15x and capital expenditure at 0.95x. Taking both bounds from the interval means the published range is the range the estimate itself supports. A whole-model re-run</t>
+          <t>beta 0.586 — the BOTTOM of the same interval — with the rate anchor at 1.15x and capital expenditure at 0.95x. Taking both bounds from the interval means the published range is the range the estimate itself supports. A whole-model re-run</t>
         </is>
       </c>
       <c r="C7" s="21" t="n">
-        <v>10.13215941638862</v>
+        <v>12.2389432347382</v>
       </c>
     </row>
     <row r="8" ht="28" customHeight="1">
@@ -8080,7 +8153,7 @@
       </c>
       <c r="B15" s="20" t="inlineStr">
         <is>
-          <t>161 weekly observations, R-squared 15.8%, standard error 0.199, 90% confidence interval 0.758 to 1.412 — the usability gate is passed, and this is the index the method asks for</t>
+          <t>159 weekly observations, R-squared 18.1%, standard error 0.315, 90% confidence interval 0.586 to 1.621 — the usability gate is passed, and this is the index the method asks for</t>
         </is>
       </c>
       <c r="C15" s="23">
@@ -8342,13 +8415,13 @@
         </is>
       </c>
       <c r="C32" s="21" t="n">
-        <v>6.302103806955713</v>
+        <v>6.226950849542018</v>
       </c>
       <c r="D32" s="21" t="n">
-        <v>4.612173662625463</v>
+        <v>4.183627650976118</v>
       </c>
       <c r="E32" s="21" t="n">
-        <v>8.85643410508878</v>
+        <v>10.54299487474104</v>
       </c>
     </row>
     <row r="33">
@@ -8363,13 +8436,13 @@
         </is>
       </c>
       <c r="C33" s="21" t="n">
-        <v>4.892938708214075</v>
+        <v>4.798904529252498</v>
       </c>
       <c r="D33" s="21" t="n">
-        <v>3.481417824283891</v>
+        <v>3.432639967125382</v>
       </c>
       <c r="E33" s="21" t="n">
-        <v>5.996520587194937</v>
+        <v>5.866633504326449</v>
       </c>
     </row>
     <row r="34">
@@ -8536,7 +8609,7 @@
         </is>
       </c>
       <c r="C14" s="29" t="n">
-        <v>1.085</v>
+        <v>1.1032</v>
       </c>
     </row>
     <row r="15">
@@ -8556,7 +8629,7 @@
         </is>
       </c>
       <c r="C16" s="29" t="n">
-        <v>0.758</v>
+        <v>0.5855</v>
       </c>
     </row>
     <row r="17">
@@ -8566,17 +8639,17 @@
         </is>
       </c>
       <c r="C17" s="29" t="n">
-        <v>1.412</v>
+        <v>1.621</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>Beta — lead-lag sum beta from the same series, one lead and two lags</t>
+          <t>Beta — the measured slope shrunk toward the market: two-thirds of it plus one-third of 1.0</t>
         </is>
       </c>
       <c r="C18" s="29" t="n">
-        <v>1.164</v>
+        <v>1.0688</v>
       </c>
     </row>
     <row r="19">
@@ -19449,7 +19522,7 @@
     <row r="125">
       <c r="A125" s="6" t="inlineStr">
         <is>
-          <t>Beta — lead-lag sum beta, one lead and two lags</t>
+          <t>Beta — the measured slope shrunk toward the market, two-thirds of it plus one-third of 1.0</t>
         </is>
       </c>
       <c r="C125" s="23">
@@ -19460,7 +19533,7 @@
     <row r="126">
       <c r="A126" s="6" t="inlineStr">
         <is>
-          <t>Cost of equity on the lead-lag sum beta</t>
+          <t>Cost of equity on the slope shrunk toward the market</t>
         </is>
       </c>
       <c r="C126" s="50">

</xml_diff>